<commit_message>
Use a single audit date field
</commit_message>
<xml_diff>
--- a/قالب ورود اطلاعات آدیت.xlsx
+++ b/قالب ورود اطلاعات آدیت.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="فرم آدیت" sheetId="1" r:id="R30de5ba3eea34689"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="فرم آدیت" sheetId="1" r:id="Rc90ed4b78a7a4261"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,8 +13,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="0%"/>
+    <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -203,7 +204,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="59">
+  <x:cellXfs count="60">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -342,6 +343,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -354,7 +358,7 @@
         <x:color rgb="FF173A12"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF96D95E"/>
         </x:patternFill>
       </x:fill>
@@ -365,7 +369,7 @@
         <x:color rgb="FFFFFFFF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF25F5C"/>
         </x:patternFill>
       </x:fill>
@@ -594,13 +598,11 @@
       </x:c>
       <x:c r="B2" s="12" t="str"/>
       <x:c r="C2" s="9" t="str">
-        <x:v>ماه</x:v>
-      </x:c>
-      <x:c r="D2" s="12" t="str"/>
-      <x:c r="E2" s="9" t="str">
-        <x:v>سال</x:v>
-      </x:c>
-      <x:c r="F2" s="12" t="str"/>
+        <x:v>تاریخ آدیت</x:v>
+      </x:c>
+      <x:c r="D2" s="59"/>
+      <x:c r="E2" s="9"/>
+      <x:c r="F2" s="12"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="9" t="str">

</xml_diff>